<commit_message>
added graphs to reports
</commit_message>
<xml_diff>
--- a/dementia_features_log.xlsx
+++ b/dementia_features_log.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -934,7 +934,357 @@
       <c r="N9" t="n">
         <v>0.56778</v>
       </c>
-      <c r="O9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-02 17:11:17</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>microphone</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>No Dementia</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>59.38</v>
+      </c>
+      <c r="E10" t="n">
+        <v>40.62</v>
+      </c>
+      <c r="F10" t="n">
+        <v>59.38</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-0.694394</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-1.158397</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.902307</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.059817</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.041608</v>
+      </c>
+      <c r="L10" t="n">
+        <v>15.210231</v>
+      </c>
+      <c r="M10" t="n">
+        <v>17.608858</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.541067</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-06 14:46:05</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>microphone</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>No Dementia</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>52.25</v>
+      </c>
+      <c r="E11" t="n">
+        <v>47.75</v>
+      </c>
+      <c r="F11" t="n">
+        <v>52.25</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.978101</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-1.041546</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.825918</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-0.042752</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.041608</v>
+      </c>
+      <c r="L11" t="n">
+        <v>12.030054</v>
+      </c>
+      <c r="M11" t="n">
+        <v>18.623452</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.630932</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-06 14:51:55</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>microphone</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>No Dementia</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>54</v>
+      </c>
+      <c r="E12" t="n">
+        <v>54</v>
+      </c>
+      <c r="F12" t="n">
+        <v>46</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.631143</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-0.814379</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.745877</v>
+      </c>
+      <c r="J12" t="n">
+        <v>-0.431578</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.041608</v>
+      </c>
+      <c r="L12" t="n">
+        <v>22.044567</v>
+      </c>
+      <c r="M12" t="n">
+        <v>20.014343</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.629057</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-06 14:58:09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>microphone</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>No Dementia</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>64.88</v>
+      </c>
+      <c r="E13" t="n">
+        <v>35.12</v>
+      </c>
+      <c r="F13" t="n">
+        <v>64.88</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.436904</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-1.723394</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2.593544</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.103279</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.041608</v>
+      </c>
+      <c r="L13" t="n">
+        <v>22.300195</v>
+      </c>
+      <c r="M13" t="n">
+        <v>14.744527</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.658359</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-06 15:02:43</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>microphone</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>No Dementia</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>54.25</v>
+      </c>
+      <c r="E14" t="n">
+        <v>54.25</v>
+      </c>
+      <c r="F14" t="n">
+        <v>45.75</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-0.044258</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-1.499789</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2.118904</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.7970739999999999</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.041608</v>
+      </c>
+      <c r="L14" t="n">
+        <v>7.800319</v>
+      </c>
+      <c r="M14" t="n">
+        <v>20.525816</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.425951</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-06 15:07:49</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>microphone</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>No Dementia</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>55.12</v>
+      </c>
+      <c r="E15" t="n">
+        <v>44.88</v>
+      </c>
+      <c r="F15" t="n">
+        <v>55.12</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.775664</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-1.371122</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1.215813</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1.35957</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.041608</v>
+      </c>
+      <c r="L15" t="n">
+        <v>10.390985</v>
+      </c>
+      <c r="M15" t="n">
+        <v>9.237351</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.6055430000000001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-10 07:57:17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>microphone</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>No Dementia</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>55.12</v>
+      </c>
+      <c r="E16" t="n">
+        <v>55.12</v>
+      </c>
+      <c r="F16" t="n">
+        <v>44.88</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1.152109</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-3.096523</v>
+      </c>
+      <c r="I16" t="n">
+        <v>16.674629</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2.594812</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.041608</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="M16" t="n">
+        <v>15.078204</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.321366</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>